<commit_message>
feat(ims): add SOP-01 Document Control, renumber SOPs to SOP-02–11, add IMS document library
- Add SOP-01-DOCUMENT-CONTROL.docx (new first SOP, ISO 9001:2015 §7.5)
- Renumber all SOPs: old SOP-01 Marketing → SOP-02, through SOP-10 Admin → SOP-11
- Add public/ims/index.html — full document library UI at preqal.org/ims/
- Regenerate REG-01 with correct SOP-01 Document Control entry
- Update seed-qms-documents.cjs to use Google Drive URLs for all 30 records
- Update generate-excel-registers.cjs with new SOP-01 + renumbered SOPs
- Supabase qms_documents: all records now point to Google Drive view URLs
</commit_message>
<xml_diff>
--- a/public/ims/REG-01-Document-Master-Register.xlsx
+++ b/public/ims/REG-01-Document-Master-Register.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="96">
   <si>
     <t>REG-01 — Document Master Register: SOPs</t>
   </si>
@@ -47,73 +47,85 @@
     <t>SOP-01</t>
   </si>
   <si>
+    <t>Document Control Procedure</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Dr. Stefan Gravesande</t>
+  </si>
+  <si>
+    <t>2026-05-08</t>
+  </si>
+  <si>
+    <t>2027-05-08</t>
+  </si>
+  <si>
+    <t>SOP-02</t>
+  </si>
+  <si>
     <t>Marketing &amp; Lead Generation</t>
   </si>
   <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Dr. Stefan Gravesande</t>
-  </si>
-  <si>
     <t>2026-05-07</t>
   </si>
   <si>
     <t>2027-05-07</t>
   </si>
   <si>
-    <t>SOP-02</t>
+    <t>SOP-03</t>
   </si>
   <si>
     <t>Lead Capture &amp; Classification</t>
   </si>
   <si>
-    <t>SOP-03</t>
+    <t>SOP-04</t>
   </si>
   <si>
     <t>Quote &amp; Proposal</t>
   </si>
   <si>
-    <t>SOP-04</t>
+    <t>SOP-05</t>
   </si>
   <si>
     <t>Contract Execution &amp; Onboarding Setup</t>
   </si>
   <si>
-    <t>SOP-05</t>
+    <t>SOP-06</t>
   </si>
   <si>
     <t>Client Onboarding</t>
   </si>
   <si>
-    <t>SOP-06</t>
+    <t>SOP-07</t>
   </si>
   <si>
     <t>Project Delivery</t>
   </si>
   <si>
-    <t>SOP-07</t>
+    <t>SOP-08</t>
   </si>
   <si>
     <t>Project Closure &amp; Handover</t>
   </si>
   <si>
-    <t>SOP-08</t>
+    <t>SOP-09</t>
   </si>
   <si>
     <t>Billing &amp; Accounts Receivable</t>
   </si>
   <si>
-    <t>SOP-09</t>
+    <t>SOP-10</t>
   </si>
   <si>
     <t>Renewal, Upsell &amp; Client Retention</t>
   </si>
   <si>
-    <t>SOP-10</t>
+    <t>SOP-11</t>
   </si>
   <si>
     <t>Admin Dashboard Operations</t>
@@ -126,12 +138,6 @@
   </si>
   <si>
     <t>Document Master Register</t>
-  </si>
-  <si>
-    <t>2026-05-08</t>
-  </si>
-  <si>
-    <t>2027-05-08</t>
   </si>
   <si>
     <t>REG-02</t>
@@ -740,7 +746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -836,41 +842,41 @@
         <v>13</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>11</v>
@@ -882,18 +888,18 @@
         <v>13</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>11</v>
@@ -905,18 +911,18 @@
         <v>13</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>11</v>
@@ -928,18 +934,18 @@
         <v>13</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>11</v>
@@ -951,18 +957,18 @@
         <v>13</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>11</v>
@@ -974,18 +980,18 @@
         <v>13</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>11</v>
@@ -997,18 +1003,18 @@
         <v>13</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>11</v>
@@ -1020,10 +1026,33 @@
         <v>13</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1051,7 +1080,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1096,10 +1125,10 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>11</v>
@@ -1111,18 +1140,18 @@
         <v>13</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>11</v>
@@ -1134,18 +1163,18 @@
         <v>13</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>11</v>
@@ -1157,18 +1186,18 @@
         <v>13</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>11</v>
@@ -1180,18 +1209,18 @@
         <v>13</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>11</v>
@@ -1203,18 +1232,18 @@
         <v>13</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>11</v>
@@ -1226,18 +1255,18 @@
         <v>13</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>11</v>
@@ -1249,10 +1278,10 @@
         <v>13</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1280,7 +1309,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1325,10 +1354,10 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>11</v>
@@ -1340,18 +1369,18 @@
         <v>13</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>11</v>
@@ -1363,18 +1392,18 @@
         <v>13</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>11</v>
@@ -1386,18 +1415,18 @@
         <v>13</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>11</v>
@@ -1409,18 +1438,18 @@
         <v>13</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>11</v>
@@ -1432,18 +1461,18 @@
         <v>13</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>11</v>
@@ -1455,18 +1484,18 @@
         <v>13</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>11</v>
@@ -1478,18 +1507,18 @@
         <v>13</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>11</v>
@@ -1501,18 +1530,18 @@
         <v>13</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>11</v>
@@ -1524,18 +1553,18 @@
         <v>13</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>11</v>
@@ -1547,18 +1576,18 @@
         <v>13</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>11</v>
@@ -1570,18 +1599,18 @@
         <v>13</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>11</v>
@@ -1593,18 +1622,18 @@
         <v>13</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>11</v>
@@ -1616,18 +1645,18 @@
         <v>13</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>11</v>
@@ -1639,10 +1668,10 @@
         <v>13</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1670,7 +1699,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1715,10 +1744,10 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>11</v>
@@ -1730,18 +1759,18 @@
         <v>13</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>11</v>
@@ -1753,18 +1782,18 @@
         <v>13</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>11</v>
@@ -1776,18 +1805,18 @@
         <v>13</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>11</v>
@@ -1799,18 +1828,18 @@
         <v>13</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>11</v>
@@ -1822,10 +1851,10 @@
         <v>13</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1853,7 +1882,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1898,10 +1927,10 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>11</v>
@@ -1913,10 +1942,10 @@
         <v>13</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>